<commit_message>
updating to reflect latest version style
</commit_message>
<xml_diff>
--- a/Patient_Distribution.xlsx
+++ b/Patient_Distribution.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7620"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7620"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -753,7 +753,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:B119"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -765,7 +764,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -773,7 +772,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -781,7 +780,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -789,7 +788,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -797,7 +796,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -805,7 +804,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -813,7 +812,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -821,7 +820,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -829,7 +828,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -837,7 +836,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -845,7 +844,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>13</v>
       </c>
@@ -853,7 +852,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>14</v>
       </c>
@@ -861,7 +860,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>15</v>
       </c>
@@ -869,7 +868,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -877,7 +876,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -885,7 +884,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>18</v>
       </c>
@@ -893,7 +892,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>19</v>
       </c>
@@ -901,7 +900,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>20</v>
       </c>
@@ -909,7 +908,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -917,7 +916,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>22</v>
       </c>
@@ -925,7 +924,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -933,7 +932,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>24</v>
       </c>
@@ -941,7 +940,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>25</v>
       </c>
@@ -949,7 +948,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>26</v>
       </c>
@@ -957,7 +956,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>27</v>
       </c>
@@ -965,7 +964,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>28</v>
       </c>
@@ -973,7 +972,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>29</v>
       </c>
@@ -981,7 +980,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>30</v>
       </c>
@@ -989,7 +988,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="30" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>31</v>
       </c>
@@ -997,7 +996,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>32</v>
       </c>
@@ -1005,7 +1004,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>33</v>
       </c>
@@ -1013,7 +1012,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="33" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>34</v>
       </c>
@@ -1021,7 +1020,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="34" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>35</v>
       </c>
@@ -1029,7 +1028,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="35" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>36</v>
       </c>
@@ -1037,7 +1036,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>37</v>
       </c>
@@ -1045,7 +1044,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>38</v>
       </c>
@@ -1053,7 +1052,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>39</v>
       </c>
@@ -1061,7 +1060,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>40</v>
       </c>
@@ -1069,7 +1068,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="40" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>42</v>
       </c>
@@ -1077,7 +1076,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="41" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>43</v>
       </c>
@@ -1085,7 +1084,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="42" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>44</v>
       </c>
@@ -1093,7 +1092,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>45</v>
       </c>
@@ -1101,7 +1100,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="44" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>46</v>
       </c>
@@ -1109,7 +1108,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="45" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>47</v>
       </c>
@@ -1117,7 +1116,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="46" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>48</v>
       </c>
@@ -1125,7 +1124,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="47" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>49</v>
       </c>
@@ -1133,7 +1132,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="48" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>50</v>
       </c>
@@ -1141,7 +1140,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="49" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>51</v>
       </c>
@@ -1149,7 +1148,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="50" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>52</v>
       </c>
@@ -1157,7 +1156,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="51" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>53</v>
       </c>
@@ -1165,7 +1164,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="52" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>54</v>
       </c>
@@ -1173,7 +1172,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="53" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>55</v>
       </c>
@@ -1181,7 +1180,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="54" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>56</v>
       </c>
@@ -1189,7 +1188,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="55" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>57</v>
       </c>
@@ -1197,7 +1196,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="56" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>58</v>
       </c>
@@ -1205,7 +1204,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="57" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>59</v>
       </c>
@@ -1213,7 +1212,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="58" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>60</v>
       </c>
@@ -1221,7 +1220,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="59" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>61</v>
       </c>
@@ -1229,7 +1228,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="60" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>62</v>
       </c>
@@ -1237,7 +1236,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="61" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>63</v>
       </c>
@@ -1245,7 +1244,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="62" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>64</v>
       </c>
@@ -1253,7 +1252,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="63" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>65</v>
       </c>
@@ -1261,7 +1260,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="64" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>66</v>
       </c>
@@ -1269,7 +1268,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="65" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>67</v>
       </c>
@@ -1277,7 +1276,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="66" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>68</v>
       </c>
@@ -1285,7 +1284,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="67" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>69</v>
       </c>
@@ -1293,7 +1292,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="68" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>70</v>
       </c>
@@ -1301,7 +1300,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="69" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>71</v>
       </c>
@@ -1309,7 +1308,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="70" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>72</v>
       </c>
@@ -1317,7 +1316,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="71" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>73</v>
       </c>
@@ -1325,7 +1324,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="72" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>74</v>
       </c>
@@ -1333,7 +1332,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="73" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>75</v>
       </c>
@@ -1341,7 +1340,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="74" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>76</v>
       </c>
@@ -1349,7 +1348,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="75" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>77</v>
       </c>
@@ -1357,7 +1356,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="76" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>78</v>
       </c>
@@ -1365,7 +1364,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="77" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>79</v>
       </c>
@@ -1373,7 +1372,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="78" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>80</v>
       </c>
@@ -1381,7 +1380,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="79" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>81</v>
       </c>
@@ -1389,7 +1388,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="80" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>82</v>
       </c>
@@ -1397,7 +1396,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="81" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>83</v>
       </c>
@@ -1405,7 +1404,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="82" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>84</v>
       </c>
@@ -1413,7 +1412,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="83" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>85</v>
       </c>
@@ -1421,7 +1420,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="84" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>86</v>
       </c>
@@ -1429,7 +1428,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="85" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>87</v>
       </c>
@@ -1437,7 +1436,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="86" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>88</v>
       </c>
@@ -1445,7 +1444,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="87" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>89</v>
       </c>
@@ -1453,7 +1452,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="88" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>90</v>
       </c>
@@ -1461,7 +1460,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="89" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>91</v>
       </c>
@@ -1469,7 +1468,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="90" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>92</v>
       </c>
@@ -1477,7 +1476,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="91" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>93</v>
       </c>
@@ -1485,7 +1484,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="92" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>94</v>
       </c>
@@ -1493,7 +1492,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="93" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>95</v>
       </c>
@@ -1501,7 +1500,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="94" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>96</v>
       </c>
@@ -1509,7 +1508,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="95" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>97</v>
       </c>
@@ -1517,7 +1516,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="96" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>98</v>
       </c>
@@ -1525,7 +1524,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="97" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>99</v>
       </c>
@@ -1533,7 +1532,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="98" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>100</v>
       </c>
@@ -1541,7 +1540,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="99" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>101</v>
       </c>
@@ -1549,7 +1548,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="100" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>102</v>
       </c>
@@ -1557,7 +1556,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="101" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>103</v>
       </c>
@@ -1565,7 +1564,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="102" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>104</v>
       </c>
@@ -1573,7 +1572,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="103" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>105</v>
       </c>
@@ -1581,7 +1580,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="104" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>106</v>
       </c>
@@ -1710,13 +1709,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B119">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="Validation"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:B119"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update paper, test figures
</commit_message>
<xml_diff>
--- a/Patient_Distribution.xlsx
+++ b/Patient_Distribution.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bmanderson\Desktop\Modular_Projects\Liver_Disease_Ablation_Segmentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Modular_Projects\Liver_Disease_Ablation_Segmentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -753,6 +753,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:B119"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -767,57 +768,57 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>118</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="B4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>46</v>
       </c>
       <c r="B5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>98</v>
       </c>
       <c r="B6" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="B7" t="s">
-        <v>3</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
         <v>3</v>
@@ -825,95 +826,95 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="B9" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>112</v>
       </c>
       <c r="B10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>86</v>
       </c>
       <c r="B11" t="s">
-        <v>3</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="B12" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>116</v>
       </c>
       <c r="B13" t="s">
-        <v>3</v>
+        <v>108</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="B14" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>107</v>
       </c>
       <c r="B15" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>17</v>
+        <v>56</v>
       </c>
       <c r="B16" t="s">
-        <v>3</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B17" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>19</v>
+        <v>122</v>
       </c>
       <c r="B18" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>20</v>
+        <v>111</v>
       </c>
       <c r="B19" t="s">
-        <v>3</v>
+        <v>108</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B20" t="s">
         <v>3</v>
@@ -921,47 +922,47 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="B21" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>23</v>
+        <v>60</v>
       </c>
       <c r="B22" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="B23" t="s">
-        <v>3</v>
+        <v>41</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="B24" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>26</v>
+        <v>82</v>
       </c>
       <c r="B25" t="s">
-        <v>3</v>
+        <v>41</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B26" t="s">
         <v>3</v>
@@ -969,119 +970,119 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="B27" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="B28" t="s">
-        <v>3</v>
+        <v>41</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="B29" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>31</v>
+        <v>120</v>
       </c>
       <c r="B30" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>32</v>
+        <v>109</v>
       </c>
       <c r="B31" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>33</v>
+        <v>71</v>
       </c>
       <c r="B32" t="s">
-        <v>3</v>
+        <v>41</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="B33" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>35</v>
+        <v>92</v>
       </c>
       <c r="B34" t="s">
-        <v>3</v>
+        <v>41</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="B35" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>37</v>
+        <v>105</v>
       </c>
       <c r="B36" t="s">
-        <v>3</v>
+        <v>41</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="B37" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>39</v>
+        <v>96</v>
       </c>
       <c r="B38" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>40</v>
+        <v>119</v>
       </c>
       <c r="B39" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>42</v>
+        <v>93</v>
       </c>
       <c r="B40" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>43</v>
+        <v>103</v>
       </c>
       <c r="B41" t="s">
         <v>41</v>
@@ -1089,31 +1090,31 @@
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="B42" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>45</v>
+        <v>79</v>
       </c>
       <c r="B43" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B44" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>47</v>
+        <v>68</v>
       </c>
       <c r="B45" t="s">
         <v>41</v>
@@ -1121,23 +1122,23 @@
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="B46" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>49</v>
+        <v>80</v>
       </c>
       <c r="B47" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="B48" t="s">
         <v>41</v>
@@ -1145,47 +1146,47 @@
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>51</v>
+        <v>23</v>
       </c>
       <c r="B49" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>85</v>
+      </c>
+      <c r="B50" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>97</v>
+      </c>
+      <c r="B51" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>115</v>
+      </c>
+      <c r="B52" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>121</v>
+      </c>
+      <c r="B53" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
         <v>52</v>
-      </c>
-      <c r="B50" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>53</v>
-      </c>
-      <c r="B51" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>54</v>
-      </c>
-      <c r="B52" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>55</v>
-      </c>
-      <c r="B53" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>56</v>
       </c>
       <c r="B54" t="s">
         <v>41</v>
@@ -1193,63 +1194,63 @@
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="B55" t="s">
-        <v>41</v>
+        <v>3</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>58</v>
+        <v>7</v>
       </c>
       <c r="B56" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="B57" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="B58" t="s">
-        <v>41</v>
+        <v>108</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>61</v>
+        <v>15</v>
       </c>
       <c r="B59" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>62</v>
+        <v>81</v>
       </c>
       <c r="B60" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>63</v>
+        <v>89</v>
       </c>
       <c r="B61" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>64</v>
+        <v>100</v>
       </c>
       <c r="B62" t="s">
         <v>41</v>
@@ -1257,71 +1258,71 @@
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>65</v>
+        <v>21</v>
       </c>
       <c r="B63" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>95</v>
+      </c>
+      <c r="B64" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>78</v>
+      </c>
+      <c r="B65" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>77</v>
+      </c>
+      <c r="B66" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>76</v>
+      </c>
+      <c r="B67" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>75</v>
+      </c>
+      <c r="B68" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>70</v>
+      </c>
+      <c r="B69" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>117</v>
+      </c>
+      <c r="B70" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
         <v>66</v>
-      </c>
-      <c r="B64" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>67</v>
-      </c>
-      <c r="B65" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>68</v>
-      </c>
-      <c r="B66" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>69</v>
-      </c>
-      <c r="B67" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>70</v>
-      </c>
-      <c r="B68" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>71</v>
-      </c>
-      <c r="B69" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>72</v>
-      </c>
-      <c r="B70" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>73</v>
       </c>
       <c r="B71" t="s">
         <v>41</v>
@@ -1329,55 +1330,55 @@
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>74</v>
+        <v>22</v>
       </c>
       <c r="B72" t="s">
-        <v>41</v>
+        <v>3</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>75</v>
+        <v>10</v>
       </c>
       <c r="B73" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>76</v>
+        <v>90</v>
       </c>
       <c r="B74" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>77</v>
+        <v>114</v>
       </c>
       <c r="B75" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="B76" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="B77" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>80</v>
+        <v>47</v>
       </c>
       <c r="B78" t="s">
         <v>41</v>
@@ -1385,15 +1386,15 @@
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>81</v>
+        <v>36</v>
       </c>
       <c r="B79" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>82</v>
+        <v>49</v>
       </c>
       <c r="B80" t="s">
         <v>41</v>
@@ -1401,31 +1402,31 @@
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>83</v>
+        <v>28</v>
       </c>
       <c r="B81" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>84</v>
+        <v>113</v>
       </c>
       <c r="B82" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>85</v>
+        <v>63</v>
       </c>
       <c r="B83" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>86</v>
+        <v>67</v>
       </c>
       <c r="B84" t="s">
         <v>41</v>
@@ -1433,39 +1434,39 @@
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>87</v>
+        <v>5</v>
       </c>
       <c r="B85" t="s">
-        <v>41</v>
+        <v>3</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>88</v>
+        <v>11</v>
       </c>
       <c r="B86" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="B87" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>90</v>
+        <v>59</v>
       </c>
       <c r="B88" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>91</v>
+        <v>51</v>
       </c>
       <c r="B89" t="s">
         <v>41</v>
@@ -1473,23 +1474,23 @@
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>92</v>
+        <v>16</v>
       </c>
       <c r="B90" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="B91" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B92" t="s">
         <v>41</v>
@@ -1497,15 +1498,15 @@
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>95</v>
+        <v>13</v>
       </c>
       <c r="B93" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>96</v>
+        <v>74</v>
       </c>
       <c r="B94" t="s">
         <v>41</v>
@@ -1513,31 +1514,31 @@
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>97</v>
+        <v>2</v>
       </c>
       <c r="B95" t="s">
-        <v>41</v>
+        <v>3</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>98</v>
+        <v>26</v>
       </c>
       <c r="B96" t="s">
-        <v>41</v>
+        <v>3</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
+        <v>12</v>
+      </c>
+      <c r="B97" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
         <v>99</v>
-      </c>
-      <c r="B97" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
-        <v>100</v>
       </c>
       <c r="B98" t="s">
         <v>41</v>
@@ -1545,174 +1546,183 @@
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>101</v>
+        <v>37</v>
       </c>
       <c r="B99" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
+        <v>55</v>
+      </c>
+      <c r="B100" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>72</v>
+      </c>
+      <c r="B101" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>69</v>
+      </c>
+      <c r="B102" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
         <v>102</v>
       </c>
-      <c r="B100" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
-        <v>103</v>
-      </c>
-      <c r="B101" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
-        <v>104</v>
-      </c>
-      <c r="B102" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
-        <v>105</v>
-      </c>
       <c r="B103" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
+        <v>45</v>
+      </c>
+      <c r="B104" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
         <v>106</v>
       </c>
-      <c r="B104" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
-        <v>107</v>
-      </c>
       <c r="B105" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>109</v>
+        <v>64</v>
       </c>
       <c r="B106" t="s">
-        <v>108</v>
+        <v>41</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>110</v>
+        <v>35</v>
       </c>
       <c r="B107" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>111</v>
+        <v>62</v>
       </c>
       <c r="B108" t="s">
-        <v>108</v>
+        <v>41</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>112</v>
+        <v>9</v>
       </c>
       <c r="B109" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>113</v>
+        <v>57</v>
       </c>
       <c r="B110" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>114</v>
+        <v>65</v>
       </c>
       <c r="B111" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>115</v>
+        <v>94</v>
       </c>
       <c r="B112" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>116</v>
+        <v>53</v>
       </c>
       <c r="B113" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>117</v>
+        <v>61</v>
       </c>
       <c r="B114" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>118</v>
+        <v>50</v>
       </c>
       <c r="B115" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>119</v>
+        <v>87</v>
       </c>
       <c r="B116" t="s">
-        <v>108</v>
+        <v>41</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>120</v>
+        <v>14</v>
       </c>
       <c r="B117" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>121</v>
+        <v>84</v>
       </c>
       <c r="B118" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>122</v>
+        <v>101</v>
       </c>
       <c r="B119" t="s">
-        <v>108</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B119"/>
+  <autoFilter ref="A1:B119">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Test"/>
+      </filters>
+    </filterColumn>
+    <sortState ref="A2:B119">
+      <sortCondition ref="A1:A119"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>